<commit_message>
fix: Ajuste en los nombres de Tabasco y Tamaulipas
</commit_message>
<xml_diff>
--- a/datasets/20261021_recontrataciones_concentrado.xlsx
+++ b/datasets/20261021_recontrataciones_concentrado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INE\Documents\reductor_dias\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8F40CE-88D7-410F-B131-DF00AD2FB588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD83CD8-9034-43C3-B52A-02FDA8956359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D3C7E6B5-2A0E-4AF2-BE80-0C96F41EC4B0}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="284">
   <si>
     <t>Distrito</t>
   </si>
@@ -647,9 +647,6 @@
     <t>Paraíso</t>
   </si>
   <si>
-    <t>Ranchería Ixtacomitán 1ra Sección</t>
-  </si>
-  <si>
     <t>Nuevo Laredo</t>
   </si>
   <si>
@@ -659,15 +656,9 @@
     <t>Río Bravo</t>
   </si>
   <si>
-    <t>H. Matamoros</t>
-  </si>
-  <si>
     <t>Ciudad Victoria</t>
   </si>
   <si>
-    <t>Ciudad Mante</t>
-  </si>
-  <si>
     <t>Tampico</t>
   </si>
   <si>
@@ -906,6 +897,18 @@
   </si>
   <si>
     <t>22</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Matamoros</t>
+  </si>
+  <si>
+    <t>El Mante</t>
+  </si>
+  <si>
+    <t>27</t>
   </si>
 </sst>
 </file>
@@ -1278,7 +1281,7 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1399,6 +1402,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2283,7 +2292,7 @@
         <v>22</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>27</v>
@@ -2311,7 +2320,7 @@
         <v>22</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>27</v>
@@ -2339,7 +2348,7 @@
         <v>22</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>27</v>
@@ -2367,7 +2376,7 @@
         <v>22</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>25</v>
@@ -2395,7 +2404,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>27</v>
@@ -2423,10 +2432,10 @@
         <v>22</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E24" s="16"/>
       <c r="F24" s="11"/>
@@ -2504,7 +2513,7 @@
     </row>
     <row r="27" spans="2:21" ht="28" x14ac:dyDescent="0.35">
       <c r="B27" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C27" s="19" t="s">
         <v>12</v>
@@ -2532,7 +2541,7 @@
     </row>
     <row r="28" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B28" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C28" s="19" t="s">
         <v>22</v>
@@ -2560,7 +2569,7 @@
     </row>
     <row r="29" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B29" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C29" s="19" t="s">
         <v>12</v>
@@ -2588,7 +2597,7 @@
     </row>
     <row r="30" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B30" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C30" s="19" t="s">
         <v>22</v>
@@ -2616,7 +2625,7 @@
     </row>
     <row r="31" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B31" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C31" s="19" t="s">
         <v>23</v>
@@ -2644,10 +2653,10 @@
     </row>
     <row r="32" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B32" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>35</v>
@@ -2672,10 +2681,10 @@
     </row>
     <row r="33" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B33" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>36</v>
@@ -2700,10 +2709,10 @@
     </row>
     <row r="34" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B34" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>36</v>
@@ -2728,10 +2737,10 @@
     </row>
     <row r="35" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B35" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>35</v>
@@ -2756,10 +2765,10 @@
     </row>
     <row r="36" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B36" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="C36" s="19" t="s">
         <v>230</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>233</v>
       </c>
       <c r="D36" s="14" t="s">
         <v>37</v>
@@ -2784,7 +2793,7 @@
     </row>
     <row r="37" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B37" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C37" s="19" t="s">
         <v>12</v>
@@ -2812,7 +2821,7 @@
     </row>
     <row r="38" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B38" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C38" s="19" t="s">
         <v>22</v>
@@ -2840,7 +2849,7 @@
     </row>
     <row r="39" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B39" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C39" s="19" t="s">
         <v>12</v>
@@ -2868,7 +2877,7 @@
     </row>
     <row r="40" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B40" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C40" s="19" t="s">
         <v>22</v>
@@ -2896,7 +2905,7 @@
     </row>
     <row r="41" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B41" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C41" s="19" t="s">
         <v>23</v>
@@ -2924,10 +2933,10 @@
     </row>
     <row r="42" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B42" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>43</v>
@@ -2952,10 +2961,10 @@
     </row>
     <row r="43" spans="2:21" ht="28" x14ac:dyDescent="0.35">
       <c r="B43" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D43" s="14" t="s">
         <v>44</v>
@@ -2980,10 +2989,10 @@
     </row>
     <row r="44" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B44" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>45</v>
@@ -3008,10 +3017,10 @@
     </row>
     <row r="45" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B45" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D45" s="14" t="s">
         <v>46</v>
@@ -3036,10 +3045,10 @@
     </row>
     <row r="46" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B46" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>47</v>
@@ -3064,10 +3073,10 @@
     </row>
     <row r="47" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B47" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>45</v>
@@ -3092,10 +3101,10 @@
     </row>
     <row r="48" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B48" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="C48" s="19" t="s">
         <v>232</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>235</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>48</v>
@@ -3120,10 +3129,10 @@
     </row>
     <row r="49" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B49" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D49" s="14" t="s">
         <v>49</v>
@@ -3148,10 +3157,10 @@
     </row>
     <row r="50" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B50" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D50" s="14" t="s">
         <v>50</v>
@@ -3176,10 +3185,10 @@
     </row>
     <row r="51" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B51" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D51" s="14" t="s">
         <v>51</v>
@@ -3204,7 +3213,7 @@
     </row>
     <row r="52" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B52" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C52" s="19" t="s">
         <v>12</v>
@@ -3232,7 +3241,7 @@
     </row>
     <row r="53" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B53" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C53" s="19" t="s">
         <v>22</v>
@@ -3260,7 +3269,7 @@
     </row>
     <row r="54" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B54" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C54" s="19" t="s">
         <v>23</v>
@@ -3288,10 +3297,10 @@
     </row>
     <row r="55" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B55" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D55" s="14" t="s">
         <v>52</v>
@@ -3316,13 +3325,13 @@
     </row>
     <row r="56" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B56" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="10"/>
@@ -3344,10 +3353,10 @@
     </row>
     <row r="57" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B57" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D57" s="14" t="s">
         <v>53</v>
@@ -3372,10 +3381,10 @@
     </row>
     <row r="58" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B58" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C58" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D58" s="14" t="s">
         <v>54</v>
@@ -3400,10 +3409,10 @@
     </row>
     <row r="59" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B59" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C59" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>53</v>
@@ -3428,10 +3437,10 @@
     </row>
     <row r="60" spans="2:21" x14ac:dyDescent="0.35">
       <c r="B60" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D60" s="14" t="s">
         <v>55</v>
@@ -3455,13 +3464,13 @@
       <c r="U60" s="10"/>
     </row>
     <row r="61" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B61" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C61" s="44" t="s">
+      <c r="B61" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C61" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="D61" s="45" t="s">
+      <c r="D61" s="47" t="s">
         <v>56</v>
       </c>
       <c r="E61" s="10"/>
@@ -3483,13 +3492,13 @@
       <c r="U61" s="10"/>
     </row>
     <row r="62" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B62" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C62" s="44" t="s">
+      <c r="B62" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C62" s="46" t="s">
         <v>22</v>
       </c>
-      <c r="D62" s="45" t="s">
+      <c r="D62" s="47" t="s">
         <v>56</v>
       </c>
       <c r="E62" s="10"/>
@@ -3511,13 +3520,13 @@
       <c r="U62" s="10"/>
     </row>
     <row r="63" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B63" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C63" s="44" t="s">
+      <c r="B63" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C63" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="D63" s="45" t="s">
+      <c r="D63" s="47" t="s">
         <v>57</v>
       </c>
       <c r="E63" s="10"/>
@@ -3539,13 +3548,13 @@
       <c r="U63" s="10"/>
     </row>
     <row r="64" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B64" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C64" s="44" t="s">
-        <v>229</v>
-      </c>
-      <c r="D64" s="45" t="s">
+      <c r="B64" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C64" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="D64" s="47" t="s">
         <v>58</v>
       </c>
       <c r="E64" s="10"/>
@@ -3567,14 +3576,14 @@
       <c r="U64" s="10"/>
     </row>
     <row r="65" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B65" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C65" s="44" t="s">
-        <v>230</v>
-      </c>
-      <c r="D65" s="45" t="s">
-        <v>272</v>
+      <c r="B65" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C65" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="D65" s="47" t="s">
+        <v>269</v>
       </c>
       <c r="E65" s="10"/>
       <c r="F65" s="10"/>
@@ -3595,13 +3604,13 @@
       <c r="U65" s="10"/>
     </row>
     <row r="66" spans="2:21" ht="28" x14ac:dyDescent="0.35">
-      <c r="B66" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C66" s="44" t="s">
+      <c r="B66" s="46" t="s">
         <v>231</v>
       </c>
-      <c r="D66" s="45" t="s">
+      <c r="C66" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="D66" s="47" t="s">
         <v>60</v>
       </c>
       <c r="E66" s="10"/>
@@ -3623,13 +3632,13 @@
       <c r="U66" s="10"/>
     </row>
     <row r="67" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B67" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C67" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="D67" s="45" t="s">
+      <c r="B67" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C67" s="46" t="s">
+        <v>229</v>
+      </c>
+      <c r="D67" s="47" t="s">
         <v>56</v>
       </c>
       <c r="E67" s="10"/>
@@ -3651,13 +3660,13 @@
       <c r="U67" s="10"/>
     </row>
     <row r="68" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B68" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C68" s="44" t="s">
-        <v>233</v>
-      </c>
-      <c r="D68" s="45" t="s">
+      <c r="B68" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C68" s="46" t="s">
+        <v>230</v>
+      </c>
+      <c r="D68" s="47" t="s">
         <v>61</v>
       </c>
       <c r="E68" s="10"/>
@@ -3679,13 +3688,13 @@
       <c r="U68" s="10"/>
     </row>
     <row r="69" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B69" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C69" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="D69" s="45" t="s">
+      <c r="B69" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C69" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="D69" s="47" t="s">
         <v>62</v>
       </c>
       <c r="E69" s="10"/>
@@ -3707,13 +3716,13 @@
       <c r="U69" s="10"/>
     </row>
     <row r="70" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B70" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C70" s="44" t="s">
-        <v>235</v>
-      </c>
-      <c r="D70" s="45" t="s">
+      <c r="B70" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C70" s="46" t="s">
+        <v>232</v>
+      </c>
+      <c r="D70" s="47" t="s">
         <v>63</v>
       </c>
       <c r="E70" s="10"/>
@@ -3735,13 +3744,13 @@
       <c r="U70" s="10"/>
     </row>
     <row r="71" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B71" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C71" s="44" t="s">
-        <v>236</v>
-      </c>
-      <c r="D71" s="48" t="s">
+      <c r="B71" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C71" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="D71" s="50" t="s">
         <v>64</v>
       </c>
       <c r="E71" s="10"/>
@@ -3763,13 +3772,13 @@
       <c r="U71" s="10"/>
     </row>
     <row r="72" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B72" s="44" t="s">
+      <c r="B72" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C72" s="46" t="s">
         <v>234</v>
       </c>
-      <c r="C72" s="44" t="s">
-        <v>237</v>
-      </c>
-      <c r="D72" s="45" t="s">
+      <c r="D72" s="47" t="s">
         <v>54</v>
       </c>
       <c r="E72" s="10"/>
@@ -3791,13 +3800,13 @@
       <c r="U72" s="10"/>
     </row>
     <row r="73" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B73" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C73" s="44" t="s">
-        <v>238</v>
-      </c>
-      <c r="D73" s="45" t="s">
+      <c r="B73" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C73" s="46" t="s">
+        <v>235</v>
+      </c>
+      <c r="D73" s="47" t="s">
         <v>65</v>
       </c>
       <c r="E73" s="10"/>
@@ -3819,13 +3828,13 @@
       <c r="U73" s="10"/>
     </row>
     <row r="74" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B74" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C74" s="44" t="s">
-        <v>273</v>
-      </c>
-      <c r="D74" s="45" t="s">
+      <c r="B74" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C74" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="D74" s="47" t="s">
         <v>59</v>
       </c>
       <c r="E74" s="10"/>
@@ -3847,13 +3856,13 @@
       <c r="U74" s="10"/>
     </row>
     <row r="75" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B75" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C75" s="44" t="s">
-        <v>274</v>
-      </c>
-      <c r="D75" s="45" t="s">
+      <c r="B75" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C75" s="46" t="s">
+        <v>271</v>
+      </c>
+      <c r="D75" s="47" t="s">
         <v>66</v>
       </c>
       <c r="E75" s="10"/>
@@ -3875,14 +3884,14 @@
       <c r="U75" s="10"/>
     </row>
     <row r="76" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B76" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C76" s="44" t="s">
-        <v>275</v>
-      </c>
-      <c r="D76" s="45" t="s">
-        <v>276</v>
+      <c r="B76" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C76" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="D76" s="47" t="s">
+        <v>273</v>
       </c>
       <c r="E76" s="10"/>
       <c r="F76" s="10"/>
@@ -3903,14 +3912,14 @@
       <c r="U76" s="10"/>
     </row>
     <row r="77" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B77" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C77" s="44" t="s">
-        <v>277</v>
-      </c>
-      <c r="D77" s="45" t="s">
-        <v>278</v>
+      <c r="B77" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C77" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="D77" s="47" t="s">
+        <v>275</v>
       </c>
       <c r="E77" s="10"/>
       <c r="F77" s="10"/>
@@ -3931,13 +3940,13 @@
       <c r="U77" s="10"/>
     </row>
     <row r="78" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B78" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C78" s="44" t="s">
-        <v>279</v>
-      </c>
-      <c r="D78" s="45" t="s">
+      <c r="B78" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C78" s="46" t="s">
+        <v>276</v>
+      </c>
+      <c r="D78" s="47" t="s">
         <v>58</v>
       </c>
       <c r="E78" s="10"/>
@@ -3959,13 +3968,13 @@
       <c r="U78" s="10"/>
     </row>
     <row r="79" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B79" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C79" s="44" t="s">
-        <v>280</v>
-      </c>
-      <c r="D79" s="45" t="s">
+      <c r="B79" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C79" s="46" t="s">
+        <v>277</v>
+      </c>
+      <c r="D79" s="47" t="s">
         <v>61</v>
       </c>
       <c r="E79" s="10"/>
@@ -3987,13 +3996,13 @@
       <c r="U79" s="10"/>
     </row>
     <row r="80" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B80" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C80" s="44" t="s">
-        <v>281</v>
-      </c>
-      <c r="D80" s="45" t="s">
+      <c r="B80" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C80" s="46" t="s">
+        <v>278</v>
+      </c>
+      <c r="D80" s="47" t="s">
         <v>58</v>
       </c>
       <c r="E80" s="10"/>
@@ -4015,13 +4024,13 @@
       <c r="U80" s="10"/>
     </row>
     <row r="81" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B81" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C81" s="46">
+      <c r="B81" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C81" s="48">
         <v>21</v>
       </c>
-      <c r="D81" s="47" t="s">
+      <c r="D81" s="49" t="s">
         <v>67</v>
       </c>
       <c r="E81" s="10"/>
@@ -4043,13 +4052,13 @@
       <c r="U81" s="10"/>
     </row>
     <row r="82" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B82" s="44" t="s">
-        <v>234</v>
-      </c>
-      <c r="C82" s="44" t="s">
-        <v>282</v>
-      </c>
-      <c r="D82" s="45" t="s">
+      <c r="B82" s="46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C82" s="46" t="s">
+        <v>279</v>
+      </c>
+      <c r="D82" s="47" t="s">
         <v>58</v>
       </c>
       <c r="E82" s="10"/>
@@ -5170,7 +5179,7 @@
         <v>6</v>
       </c>
       <c r="D122" s="14" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E122" s="10"/>
       <c r="F122" s="10"/>
@@ -5450,7 +5459,7 @@
         <v>16</v>
       </c>
       <c r="D132" s="14" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E132" s="10"/>
       <c r="F132" s="10"/>
@@ -5506,7 +5515,7 @@
         <v>18</v>
       </c>
       <c r="D134" s="14" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E134" s="10"/>
       <c r="F134" s="10"/>
@@ -5534,7 +5543,7 @@
         <v>19</v>
       </c>
       <c r="D135" s="14" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E135" s="10"/>
       <c r="F135" s="10"/>
@@ -5590,7 +5599,7 @@
         <v>1</v>
       </c>
       <c r="D137" s="14" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E137" s="10"/>
       <c r="F137" s="10"/>
@@ -5674,7 +5683,7 @@
         <v>4</v>
       </c>
       <c r="D140" s="14" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E140" s="10"/>
       <c r="F140" s="10"/>
@@ -5702,7 +5711,7 @@
         <v>5</v>
       </c>
       <c r="D141" s="14" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E141" s="10"/>
       <c r="F141" s="10"/>
@@ -5730,7 +5739,7 @@
         <v>6</v>
       </c>
       <c r="D142" s="14" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E142" s="10"/>
       <c r="F142" s="10"/>
@@ -5786,7 +5795,7 @@
         <v>8</v>
       </c>
       <c r="D144" s="14" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E144" s="10"/>
       <c r="F144" s="10"/>
@@ -6738,7 +6747,7 @@
         <v>22</v>
       </c>
       <c r="D178" s="14" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E178" s="10"/>
       <c r="F178" s="10"/>
@@ -6766,7 +6775,7 @@
         <v>23</v>
       </c>
       <c r="D179" s="14" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E179" s="10"/>
       <c r="F179" s="10"/>
@@ -6791,10 +6800,10 @@
         <v>16</v>
       </c>
       <c r="C180" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D180" s="14" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E180" s="10"/>
       <c r="F180" s="10"/>
@@ -6819,10 +6828,10 @@
         <v>16</v>
       </c>
       <c r="C181" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D181" s="14" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="E181" s="10"/>
       <c r="F181" s="10"/>
@@ -6847,10 +6856,10 @@
         <v>16</v>
       </c>
       <c r="C182" s="19" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D182" s="14" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E182" s="10"/>
       <c r="F182" s="10"/>
@@ -6875,7 +6884,7 @@
         <v>16</v>
       </c>
       <c r="C183" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D183" s="14" t="s">
         <v>135</v>
@@ -6903,7 +6912,7 @@
         <v>16</v>
       </c>
       <c r="C184" s="19" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D184" s="14" t="s">
         <v>136</v>
@@ -6931,10 +6940,10 @@
         <v>16</v>
       </c>
       <c r="C185" s="19" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D185" s="14" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E185" s="10"/>
       <c r="F185" s="10"/>
@@ -6959,7 +6968,7 @@
         <v>16</v>
       </c>
       <c r="C186" s="19" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D186" s="14" t="s">
         <v>136</v>
@@ -6987,7 +6996,7 @@
         <v>16</v>
       </c>
       <c r="C187" s="19" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D187" s="14" t="s">
         <v>137</v>
@@ -7099,7 +7108,7 @@
         <v>17</v>
       </c>
       <c r="C191" s="19" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D191" s="14" t="s">
         <v>141</v>
@@ -7127,7 +7136,7 @@
         <v>17</v>
       </c>
       <c r="C192" s="19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D192" s="14" t="s">
         <v>142</v>
@@ -7298,7 +7307,7 @@
         <v>23</v>
       </c>
       <c r="D198" s="14" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E198" s="10"/>
       <c r="F198" s="10"/>
@@ -7323,7 +7332,7 @@
         <v>19</v>
       </c>
       <c r="C199" s="10" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="D199" s="14" t="s">
         <v>148</v>
@@ -7351,7 +7360,7 @@
         <v>19</v>
       </c>
       <c r="C200" s="10" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D200" s="14" t="s">
         <v>149</v>
@@ -7379,7 +7388,7 @@
         <v>19</v>
       </c>
       <c r="C201" s="10" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D201" s="14" t="s">
         <v>149</v>
@@ -7407,10 +7416,10 @@
         <v>19</v>
       </c>
       <c r="C202" s="10" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D202" s="14" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E202" s="10"/>
       <c r="F202" s="10"/>
@@ -7435,7 +7444,7 @@
         <v>19</v>
       </c>
       <c r="C203" s="10" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D203" s="14" t="s">
         <v>150</v>
@@ -7463,7 +7472,7 @@
         <v>19</v>
       </c>
       <c r="C204" s="10" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D204" s="14" t="s">
         <v>151</v>
@@ -7690,7 +7699,7 @@
         <v>3</v>
       </c>
       <c r="D212" s="14" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E212" s="10"/>
       <c r="F212" s="10"/>
@@ -7774,7 +7783,7 @@
         <v>6</v>
       </c>
       <c r="D215" s="14" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E215" s="10"/>
       <c r="F215" s="10"/>
@@ -7858,7 +7867,7 @@
         <v>9</v>
       </c>
       <c r="D218" s="14" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E218" s="10"/>
       <c r="F218" s="10"/>
@@ -7914,7 +7923,7 @@
         <v>1</v>
       </c>
       <c r="D220" s="14" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E220" s="10"/>
       <c r="F220" s="10"/>
@@ -7970,7 +7979,7 @@
         <v>3</v>
       </c>
       <c r="D222" s="14" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E222" s="10"/>
       <c r="F222" s="10"/>
@@ -8026,7 +8035,7 @@
         <v>5</v>
       </c>
       <c r="D224" s="14" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E224" s="10"/>
       <c r="F224" s="10"/>
@@ -8054,7 +8063,7 @@
         <v>6</v>
       </c>
       <c r="D225" s="14" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E225" s="10"/>
       <c r="F225" s="10"/>
@@ -8138,7 +8147,7 @@
         <v>9</v>
       </c>
       <c r="D228" s="14" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E228" s="10"/>
       <c r="F228" s="10"/>
@@ -8166,7 +8175,7 @@
         <v>10</v>
       </c>
       <c r="D229" s="14" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="E229" s="10"/>
       <c r="F229" s="10"/>
@@ -8194,7 +8203,7 @@
         <v>11</v>
       </c>
       <c r="D230" s="14" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E230" s="10"/>
       <c r="F230" s="10"/>
@@ -8222,7 +8231,7 @@
         <v>12</v>
       </c>
       <c r="D231" s="14" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E231" s="10"/>
       <c r="F231" s="10"/>
@@ -8641,7 +8650,7 @@
       <c r="C246" s="19">
         <v>1</v>
       </c>
-      <c r="D246" s="43" t="s">
+      <c r="D246" s="45" t="s">
         <v>179</v>
       </c>
       <c r="E246" s="10"/>
@@ -8669,7 +8678,7 @@
       <c r="C247" s="19">
         <v>2</v>
       </c>
-      <c r="D247" s="43" t="s">
+      <c r="D247" s="45" t="s">
         <v>176</v>
       </c>
       <c r="E247" s="10"/>
@@ -8697,7 +8706,7 @@
       <c r="C248" s="19">
         <v>3</v>
       </c>
-      <c r="D248" s="43" t="s">
+      <c r="D248" s="45" t="s">
         <v>177</v>
       </c>
       <c r="E248" s="10"/>
@@ -8725,7 +8734,7 @@
       <c r="C249" s="19">
         <v>4</v>
       </c>
-      <c r="D249" s="43" t="s">
+      <c r="D249" s="45" t="s">
         <v>178</v>
       </c>
       <c r="E249" s="10"/>
@@ -8753,7 +8762,7 @@
       <c r="C250" s="19">
         <v>5</v>
       </c>
-      <c r="D250" s="43" t="s">
+      <c r="D250" s="45" t="s">
         <v>179</v>
       </c>
       <c r="E250" s="10"/>
@@ -8781,7 +8790,7 @@
       <c r="C251" s="19">
         <v>6</v>
       </c>
-      <c r="D251" s="43" t="s">
+      <c r="D251" s="45" t="s">
         <v>179</v>
       </c>
       <c r="E251" s="10"/>
@@ -8809,7 +8818,7 @@
       <c r="C252" s="19">
         <v>7</v>
       </c>
-      <c r="D252" s="43" t="s">
+      <c r="D252" s="45" t="s">
         <v>180</v>
       </c>
       <c r="E252" s="10"/>
@@ -8950,7 +8959,7 @@
         <v>5</v>
       </c>
       <c r="D257" s="14" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E257" s="10"/>
       <c r="F257" s="10"/>
@@ -9006,7 +9015,7 @@
         <v>7</v>
       </c>
       <c r="D259" s="14" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E259" s="10"/>
       <c r="F259" s="10"/>
@@ -9223,13 +9232,13 @@
       <c r="U266" s="10"/>
     </row>
     <row r="267" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B267" s="19">
-        <v>27</v>
-      </c>
-      <c r="C267" s="19">
-        <v>1</v>
-      </c>
-      <c r="D267" s="14" t="s">
+      <c r="B267" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C267" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="D267" s="47" t="s">
         <v>191</v>
       </c>
       <c r="E267" s="10"/>
@@ -9251,13 +9260,13 @@
       <c r="U267" s="10"/>
     </row>
     <row r="268" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B268" s="19">
-        <v>27</v>
-      </c>
-      <c r="C268" s="19">
-        <v>2</v>
-      </c>
-      <c r="D268" s="14" t="s">
+      <c r="B268" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C268" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="D268" s="47" t="s">
         <v>192</v>
       </c>
       <c r="E268" s="10"/>
@@ -9279,13 +9288,13 @@
       <c r="U268" s="10"/>
     </row>
     <row r="269" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B269" s="19">
-        <v>27</v>
-      </c>
-      <c r="C269" s="19">
-        <v>3</v>
-      </c>
-      <c r="D269" s="14" t="s">
+      <c r="B269" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C269" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="D269" s="47" t="s">
         <v>193</v>
       </c>
       <c r="E269" s="10"/>
@@ -9307,13 +9316,13 @@
       <c r="U269" s="10"/>
     </row>
     <row r="270" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B270" s="19">
-        <v>27</v>
-      </c>
-      <c r="C270" s="19">
-        <v>4</v>
-      </c>
-      <c r="D270" s="14" t="s">
+      <c r="B270" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C270" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="D270" s="47" t="s">
         <v>194</v>
       </c>
       <c r="E270" s="10"/>
@@ -9335,13 +9344,13 @@
       <c r="U270" s="10"/>
     </row>
     <row r="271" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B271" s="19">
-        <v>27</v>
-      </c>
-      <c r="C271" s="19">
-        <v>5</v>
-      </c>
-      <c r="D271" s="14" t="s">
+      <c r="B271" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C271" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="D271" s="47" t="s">
         <v>195</v>
       </c>
       <c r="E271" s="10"/>
@@ -9362,15 +9371,15 @@
       <c r="T271" s="10"/>
       <c r="U271" s="10"/>
     </row>
-    <row r="272" spans="2:21" ht="28" x14ac:dyDescent="0.35">
-      <c r="B272" s="19">
-        <v>27</v>
-      </c>
-      <c r="C272" s="19">
-        <v>6</v>
-      </c>
-      <c r="D272" s="14" t="s">
-        <v>196</v>
+    <row r="272" spans="2:21" x14ac:dyDescent="0.35">
+      <c r="B272" s="46" t="s">
+        <v>283</v>
+      </c>
+      <c r="C272" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="D272" s="47" t="s">
+        <v>194</v>
       </c>
       <c r="E272" s="10"/>
       <c r="F272" s="10"/>
@@ -9391,14 +9400,14 @@
       <c r="U272" s="10"/>
     </row>
     <row r="273" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B273" s="19">
-        <v>28</v>
-      </c>
-      <c r="C273" s="19">
-        <v>1</v>
-      </c>
-      <c r="D273" s="14" t="s">
-        <v>197</v>
+      <c r="B273" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C273" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="D273" s="47" t="s">
+        <v>196</v>
       </c>
       <c r="E273" s="10"/>
       <c r="F273" s="10"/>
@@ -9419,14 +9428,14 @@
       <c r="U273" s="10"/>
     </row>
     <row r="274" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B274" s="19">
-        <v>28</v>
-      </c>
-      <c r="C274" s="19">
-        <v>2</v>
-      </c>
-      <c r="D274" s="14" t="s">
-        <v>198</v>
+      <c r="B274" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C274" s="46" t="s">
+        <v>22</v>
+      </c>
+      <c r="D274" s="47" t="s">
+        <v>197</v>
       </c>
       <c r="E274" s="10"/>
       <c r="F274" s="10"/>
@@ -9447,14 +9456,14 @@
       <c r="U274" s="10"/>
     </row>
     <row r="275" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B275" s="19">
-        <v>28</v>
-      </c>
-      <c r="C275" s="19">
-        <v>3</v>
-      </c>
-      <c r="D275" s="14" t="s">
-        <v>199</v>
+      <c r="B275" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C275" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="D275" s="47" t="s">
+        <v>198</v>
       </c>
       <c r="E275" s="10"/>
       <c r="F275" s="10"/>
@@ -9475,14 +9484,14 @@
       <c r="U275" s="10"/>
     </row>
     <row r="276" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B276" s="19">
-        <v>28</v>
-      </c>
-      <c r="C276" s="19">
-        <v>4</v>
-      </c>
-      <c r="D276" s="14" t="s">
-        <v>200</v>
+      <c r="B276" s="43" t="s">
+        <v>280</v>
+      </c>
+      <c r="C276" s="43" t="s">
+        <v>226</v>
+      </c>
+      <c r="D276" s="44" t="s">
+        <v>281</v>
       </c>
       <c r="E276" s="10"/>
       <c r="F276" s="10"/>
@@ -9503,14 +9512,14 @@
       <c r="U276" s="10"/>
     </row>
     <row r="277" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B277" s="19">
-        <v>28</v>
-      </c>
-      <c r="C277" s="19">
-        <v>5</v>
-      </c>
-      <c r="D277" s="14" t="s">
-        <v>201</v>
+      <c r="B277" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C277" s="46" t="s">
+        <v>227</v>
+      </c>
+      <c r="D277" s="47" t="s">
+        <v>199</v>
       </c>
       <c r="E277" s="10"/>
       <c r="F277" s="10"/>
@@ -9531,14 +9540,14 @@
       <c r="U277" s="10"/>
     </row>
     <row r="278" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B278" s="19">
-        <v>28</v>
-      </c>
-      <c r="C278" s="19">
-        <v>6</v>
-      </c>
-      <c r="D278" s="14" t="s">
-        <v>202</v>
+      <c r="B278" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C278" s="46" t="s">
+        <v>228</v>
+      </c>
+      <c r="D278" s="47" t="s">
+        <v>282</v>
       </c>
       <c r="E278" s="10"/>
       <c r="F278" s="10"/>
@@ -9559,14 +9568,14 @@
       <c r="U278" s="10"/>
     </row>
     <row r="279" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B279" s="19">
-        <v>28</v>
-      </c>
-      <c r="C279" s="19">
-        <v>7</v>
-      </c>
-      <c r="D279" s="14" t="s">
-        <v>198</v>
+      <c r="B279" s="43" t="s">
+        <v>280</v>
+      </c>
+      <c r="C279" s="43" t="s">
+        <v>229</v>
+      </c>
+      <c r="D279" s="44" t="s">
+        <v>197</v>
       </c>
       <c r="E279" s="10"/>
       <c r="F279" s="10"/>
@@ -9587,14 +9596,14 @@
       <c r="U279" s="10"/>
     </row>
     <row r="280" spans="2:21" x14ac:dyDescent="0.35">
-      <c r="B280" s="19">
-        <v>28</v>
-      </c>
-      <c r="C280" s="19">
-        <v>8</v>
-      </c>
-      <c r="D280" s="14" t="s">
-        <v>203</v>
+      <c r="B280" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="C280" s="46" t="s">
+        <v>230</v>
+      </c>
+      <c r="D280" s="47" t="s">
+        <v>200</v>
       </c>
       <c r="E280" s="10"/>
       <c r="F280" s="10"/>
@@ -9622,7 +9631,7 @@
         <v>12</v>
       </c>
       <c r="D281" s="14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="E281" s="10"/>
       <c r="F281" s="10"/>
@@ -9650,7 +9659,7 @@
         <v>22</v>
       </c>
       <c r="D282" s="14" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E282" s="10"/>
       <c r="F282" s="10"/>
@@ -9678,7 +9687,7 @@
         <v>23</v>
       </c>
       <c r="D283" s="14" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E283" s="10"/>
       <c r="F283" s="10"/>
@@ -9706,7 +9715,7 @@
         <v>1</v>
       </c>
       <c r="D284" s="14" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E284" s="10"/>
       <c r="F284" s="10"/>
@@ -9734,7 +9743,7 @@
         <v>2</v>
       </c>
       <c r="D285" s="14" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E285" s="10"/>
       <c r="F285" s="10"/>
@@ -9762,7 +9771,7 @@
         <v>3</v>
       </c>
       <c r="D286" s="14" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E286" s="10"/>
       <c r="F286" s="10"/>
@@ -9790,7 +9799,7 @@
         <v>4</v>
       </c>
       <c r="D287" s="14" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E287" s="10"/>
       <c r="F287" s="10"/>
@@ -9818,7 +9827,7 @@
         <v>5</v>
       </c>
       <c r="D288" s="14" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E288" s="10"/>
       <c r="F288" s="10"/>
@@ -9846,7 +9855,7 @@
         <v>6</v>
       </c>
       <c r="D289" s="14" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E289" s="10"/>
       <c r="F289" s="10"/>
@@ -9874,7 +9883,7 @@
         <v>7</v>
       </c>
       <c r="D290" s="14" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E290" s="10"/>
       <c r="F290" s="10"/>
@@ -9902,7 +9911,7 @@
         <v>8</v>
       </c>
       <c r="D291" s="14" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E291" s="10"/>
       <c r="F291" s="10"/>
@@ -9930,7 +9939,7 @@
         <v>9</v>
       </c>
       <c r="D292" s="14" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E292" s="10"/>
       <c r="F292" s="10"/>
@@ -9958,7 +9967,7 @@
         <v>10</v>
       </c>
       <c r="D293" s="14" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E293" s="10"/>
       <c r="F293" s="10"/>
@@ -9986,7 +9995,7 @@
         <v>11</v>
       </c>
       <c r="D294" s="14" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E294" s="10"/>
       <c r="F294" s="10"/>
@@ -10014,7 +10023,7 @@
         <v>12</v>
       </c>
       <c r="D295" s="14" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E295" s="10"/>
       <c r="F295" s="10"/>
@@ -10042,7 +10051,7 @@
         <v>13</v>
       </c>
       <c r="D296" s="14" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E296" s="10"/>
       <c r="F296" s="10"/>
@@ -10070,7 +10079,7 @@
         <v>14</v>
       </c>
       <c r="D297" s="14" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E297" s="10"/>
       <c r="F297" s="10"/>
@@ -10098,7 +10107,7 @@
         <v>15</v>
       </c>
       <c r="D298" s="14" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E298" s="10"/>
       <c r="F298" s="10"/>
@@ -10126,7 +10135,7 @@
         <v>16</v>
       </c>
       <c r="D299" s="14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E299" s="10"/>
       <c r="F299" s="10"/>
@@ -10154,7 +10163,7 @@
         <v>17</v>
       </c>
       <c r="D300" s="14" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E300" s="10"/>
       <c r="F300" s="10"/>
@@ -10182,7 +10191,7 @@
         <v>18</v>
       </c>
       <c r="D301" s="14" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E301" s="10"/>
       <c r="F301" s="10"/>
@@ -10210,7 +10219,7 @@
         <v>19</v>
       </c>
       <c r="D302" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E302" s="10"/>
       <c r="F302" s="10"/>
@@ -10238,7 +10247,7 @@
         <v>1</v>
       </c>
       <c r="D303" s="14" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E303" s="10"/>
       <c r="F303" s="10"/>
@@ -10266,7 +10275,7 @@
         <v>2</v>
       </c>
       <c r="D304" s="14" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E304" s="10"/>
       <c r="F304" s="10"/>
@@ -10294,7 +10303,7 @@
         <v>3</v>
       </c>
       <c r="D305" s="14" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E305" s="10"/>
       <c r="F305" s="10"/>
@@ -10322,7 +10331,7 @@
         <v>4</v>
       </c>
       <c r="D306" s="14" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E306" s="10"/>
       <c r="F306" s="10"/>
@@ -10350,7 +10359,7 @@
         <v>5</v>
       </c>
       <c r="D307" s="14" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E307" s="10"/>
       <c r="F307" s="10"/>
@@ -10378,7 +10387,7 @@
         <v>6</v>
       </c>
       <c r="D308" s="14" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E308" s="10"/>
       <c r="F308" s="10"/>
@@ -10406,7 +10415,7 @@
         <v>1</v>
       </c>
       <c r="D309" s="14" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="E309" s="10"/>
       <c r="F309" s="10"/>
@@ -10434,7 +10443,7 @@
         <v>2</v>
       </c>
       <c r="D310" s="14" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E310" s="10"/>
       <c r="F310" s="10"/>
@@ -10462,7 +10471,7 @@
         <v>3</v>
       </c>
       <c r="D311" s="14" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E311" s="10"/>
       <c r="F311" s="10"/>

</xml_diff>